<commit_message>
Add M3 quality tests, server fixes and traceability evidence
</commit_message>
<xml_diff>
--- a/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
+++ b/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Person 2 RTM" sheetId="1" r:id="R889ce99fadd84655"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Person 2 RTM" sheetId="1" r:id="Rf43969e42baa4807"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34,7 +34,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -51,6 +51,16 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC2E7F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -58,7 +68,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -84,6 +94,12 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -326,6 +342,10 @@
     <x:col min="13" max="13" width="46" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="34" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="40" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="62" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="62" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="62" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="62" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2">
@@ -389,6 +409,18 @@
       <x:c r="O6" s="8" t="str">
         <x:v>GitHub evidence</x:v>
       </x:c>
+      <x:c r="P6" s="8" t="str">
+        <x:v>M3 test cases</x:v>
+      </x:c>
+      <x:c r="Q6" s="8" t="str">
+        <x:v>M3 expected result</x:v>
+      </x:c>
+      <x:c r="R6" s="8" t="str">
+        <x:v>M3 actual evidence</x:v>
+      </x:c>
+      <x:c r="S6" s="8" t="str">
+        <x:v>M3 defects and acceptance status</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="95" customHeight="1">
       <x:c r="A7" s="4" t="str">
@@ -438,6 +470,18 @@
       <x:c r="O7" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P7" s="11" t="str">
+        <x:v>T23, M3-S01</x:v>
+      </x:c>
+      <x:c r="Q7" s="11" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T23, M3-S01</x:v>
+      </x:c>
+      <x:c r="R7" s="11" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S7" s="11" t="str">
+        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="95" customHeight="1">
       <x:c r="A8" s="4" t="str">
@@ -487,6 +531,18 @@
       <x:c r="O8" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P8" s="12" t="str">
+        <x:v>T01, T02, T21, T23, M3-U01, M3-U02, M3-S01, M3-S02</x:v>
+      </x:c>
+      <x:c r="Q8" s="12" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T01, T02, T21, T23, M3-U01, M3-U02, M3-S01, M3-S02</x:v>
+      </x:c>
+      <x:c r="R8" s="12" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S8" s="12" t="str">
+        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="95" customHeight="1">
       <x:c r="A9" s="4" t="str">
@@ -536,6 +592,18 @@
       <x:c r="O9" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P9" s="11" t="str">
+        <x:v>T02, T03</x:v>
+      </x:c>
+      <x:c r="Q9" s="11" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T02, T03</x:v>
+      </x:c>
+      <x:c r="R9" s="11" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S9" s="11" t="str">
+        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="95" customHeight="1">
       <x:c r="A10" s="4" t="str">
@@ -585,6 +653,18 @@
       <x:c r="O10" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P10" s="12" t="str">
+        <x:v>T04, M3-S02</x:v>
+      </x:c>
+      <x:c r="Q10" s="12" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T04, M3-S02</x:v>
+      </x:c>
+      <x:c r="R10" s="12" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S10" s="12" t="str">
+        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="95" customHeight="1">
       <x:c r="A11" s="4" t="str">
@@ -634,6 +714,18 @@
       <x:c r="O11" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P11" s="11" t="str">
+        <x:v>T09, M3-S01</x:v>
+      </x:c>
+      <x:c r="Q11" s="11" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T09, M3-S01</x:v>
+      </x:c>
+      <x:c r="R11" s="11" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S11" s="11" t="str">
+        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="95" customHeight="1">
       <x:c r="A12" s="4" t="str">
@@ -683,6 +775,18 @@
       <x:c r="O12" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P12" s="12" t="str">
+        <x:v>T05, M3-S02</x:v>
+      </x:c>
+      <x:c r="Q12" s="12" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T05, M3-S02</x:v>
+      </x:c>
+      <x:c r="R12" s="12" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S12" s="12" t="str">
+        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="95" customHeight="1">
       <x:c r="A13" s="4" t="str">
@@ -732,6 +836,18 @@
       <x:c r="O13" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P13" s="11" t="str">
+        <x:v>T14, T16</x:v>
+      </x:c>
+      <x:c r="Q13" s="11" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T14, T16</x:v>
+      </x:c>
+      <x:c r="R13" s="11" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S13" s="11" t="str">
+        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="95" customHeight="1">
       <x:c r="A14" s="4" t="str">
@@ -750,7 +866,7 @@
       </x:c>
       <x:c r="E14" s="4" t="inlineStr">
         <x:is>
-          <x:t>AC-F08: Assignment locks the ticket to one category-authorised owner. Ineligible owners or missing due dates abort the assignment. Reassignment preserves the prior owner in the history log and notifies the requester.</x:t>
+          <x:t xml:space="preserve">AC-F08: Assignment locks the ticket to one category-authorised owner. Ineligible owners or missing due dates abort the assignment. Reassignment preserves the prior owner in the history log and notifies the requester.</x:t>
         </x:is>
       </x:c>
       <x:c r="F14" s="4" t="str">
@@ -782,6 +898,18 @@
       </x:c>
       <x:c r="O14" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
+      </x:c>
+      <x:c r="P14" s="12" t="str">
+        <x:v>T06, T20, M3-S01</x:v>
+      </x:c>
+      <x:c r="Q14" s="12" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T06, T20, M3-S01</x:v>
+      </x:c>
+      <x:c r="R14" s="12" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S14" s="12" t="str">
+        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="95" customHeight="1">
@@ -832,6 +960,18 @@
       <x:c r="O15" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P15" s="11" t="str">
+        <x:v>T19, M3-U03, M3-U06</x:v>
+      </x:c>
+      <x:c r="Q15" s="11" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T19, M3-U03, M3-U06</x:v>
+      </x:c>
+      <x:c r="R15" s="11" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S15" s="11" t="str">
+        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="95" customHeight="1">
       <x:c r="A16" s="4" t="str">
@@ -881,6 +1021,18 @@
       <x:c r="O16" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P16" s="12" t="str">
+        <x:v>T07, T08, M3-U05, M3-S01, M3-S02</x:v>
+      </x:c>
+      <x:c r="Q16" s="12" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T07, T08, M3-U05, M3-S01, M3-S02</x:v>
+      </x:c>
+      <x:c r="R16" s="12" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S16" s="12" t="str">
+        <x:v>DEF-M3-005; browser reasons pending</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="95" customHeight="1">
       <x:c r="A17" s="4" t="str">
@@ -930,6 +1082,18 @@
       <x:c r="O17" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P17" s="11" t="str">
+        <x:v>T09, T24, M3-S01</x:v>
+      </x:c>
+      <x:c r="Q17" s="11" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T09, T24, M3-S01</x:v>
+      </x:c>
+      <x:c r="R17" s="11" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S17" s="11" t="str">
+        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="95" customHeight="1">
       <x:c r="A18" s="4" t="str">
@@ -979,6 +1143,18 @@
       <x:c r="O18" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P18" s="12" t="str">
+        <x:v>T13, T15, T16</x:v>
+      </x:c>
+      <x:c r="Q18" s="12" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T13, T15, T16</x:v>
+      </x:c>
+      <x:c r="R18" s="12" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S18" s="12" t="str">
+        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="95" customHeight="1">
       <x:c r="A19" s="4" t="str">
@@ -1028,6 +1204,18 @@
       <x:c r="O19" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P19" s="11" t="str">
+        <x:v>T11, T12, T19, T20</x:v>
+      </x:c>
+      <x:c r="Q19" s="11" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T11, T12, T19, T20</x:v>
+      </x:c>
+      <x:c r="R19" s="11" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S19" s="11" t="str">
+        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="95" customHeight="1">
       <x:c r="A20" s="4" t="str">
@@ -1052,7 +1240,7 @@
       </x:c>
       <x:c r="G20" s="4" t="inlineStr">
         <x:is>
-          <x:t>users.role, requester_id and staff_categories authorisation</x:t>
+          <x:t xml:space="preserve">users.role, requester_id and staff_categories authorisation</x:t>
         </x:is>
       </x:c>
       <x:c r="H20" s="4" t="str">
@@ -1078,6 +1266,18 @@
       </x:c>
       <x:c r="O20" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
+      </x:c>
+      <x:c r="P20" s="12" t="str">
+        <x:v>T04, T05, T13, T22, T23, M3-I01</x:v>
+      </x:c>
+      <x:c r="Q20" s="12" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T04, T05, T13, T22, T23, M3-I01</x:v>
+      </x:c>
+      <x:c r="R20" s="12" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S20" s="12" t="str">
+        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="95" customHeight="1">
@@ -1106,7 +1306,7 @@
       </x:c>
       <x:c r="H21" s="4" t="inlineStr">
         <x:is>
-          <x:t>HTTPS proposed; Secure cookie option; sanitised errors</x:t>
+          <x:t xml:space="preserve">HTTPS proposed; Secure cookie option; sanitised errors</x:t>
         </x:is>
       </x:c>
       <x:c r="I21" s="4" t="str">
@@ -1129,6 +1329,18 @@
       </x:c>
       <x:c r="O21" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
+      </x:c>
+      <x:c r="P21" s="11" t="str">
+        <x:v>T21, M3-I01, M3-I02</x:v>
+      </x:c>
+      <x:c r="Q21" s="11" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T21, M3-I01, M3-I02</x:v>
+      </x:c>
+      <x:c r="R21" s="11" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S21" s="11" t="str">
+        <x:v>DEF-M3-002 fixed locally; TLS/secret scan pending</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="95" customHeight="1">
@@ -1179,6 +1391,18 @@
       <x:c r="O22" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P22" s="12" t="str">
+        <x:v>T10, T11, T17, M3-U04, M3-S02</x:v>
+      </x:c>
+      <x:c r="Q22" s="12" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T10, T11, T17, M3-U04, M3-S02</x:v>
+      </x:c>
+      <x:c r="R22" s="12" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S22" s="12" t="str">
+        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="95" customHeight="1">
       <x:c r="A23" s="4" t="str">
@@ -1228,6 +1452,18 @@
       <x:c r="O23" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P23" s="11" t="str">
+        <x:v>No additional automated acceptance evidence</x:v>
+      </x:c>
+      <x:c r="Q23" s="11" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows No additional automated acceptance evidence</x:v>
+      </x:c>
+      <x:c r="R23" s="11" t="str">
+        <x:v>No qualifying local automation result</x:v>
+      </x:c>
+      <x:c r="S23" s="11" t="str">
+        <x:v>Operational/quality acceptance pending</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="95" customHeight="1">
       <x:c r="A24" s="4" t="str">
@@ -1276,6 +1512,18 @@
       </x:c>
       <x:c r="O24" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
+      </x:c>
+      <x:c r="P24" s="12" t="str">
+        <x:v>No additional automated acceptance evidence</x:v>
+      </x:c>
+      <x:c r="Q24" s="12" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows No additional automated acceptance evidence</x:v>
+      </x:c>
+      <x:c r="R24" s="12" t="str">
+        <x:v>No qualifying local automation result</x:v>
+      </x:c>
+      <x:c r="S24" s="12" t="str">
+        <x:v>Operational/quality acceptance pending</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="95" customHeight="1">
@@ -1327,6 +1575,18 @@
       <x:c r="O25" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P25" s="11" t="str">
+        <x:v>No additional automated acceptance evidence</x:v>
+      </x:c>
+      <x:c r="Q25" s="11" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows No additional automated acceptance evidence</x:v>
+      </x:c>
+      <x:c r="R25" s="11" t="str">
+        <x:v>No qualifying local automation result</x:v>
+      </x:c>
+      <x:c r="S25" s="11" t="str">
+        <x:v>Operational/quality acceptance pending</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="95" customHeight="1">
       <x:c r="A26" s="4" t="str">
@@ -1351,7 +1611,7 @@
       </x:c>
       <x:c r="G26" s="4" t="inlineStr">
         <x:is>
-          <x:t>Database health query; sanitised failure metadata</x:t>
+          <x:t xml:space="preserve">Database health query; sanitised failure metadata</x:t>
         </x:is>
       </x:c>
       <x:c r="H26" s="4" t="str">
@@ -1377,6 +1637,18 @@
       </x:c>
       <x:c r="O26" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
+      </x:c>
+      <x:c r="P26" s="12" t="str">
+        <x:v>M3-I03</x:v>
+      </x:c>
+      <x:c r="Q26" s="12" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows M3-I03</x:v>
+      </x:c>
+      <x:c r="R26" s="12" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S26" s="12" t="str">
+        <x:v>Operational/quality acceptance pending</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="95" customHeight="1">
@@ -1427,11 +1699,23 @@
       <x:c r="O27" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
+      <x:c r="P27" s="11" t="str">
+        <x:v>T18</x:v>
+      </x:c>
+      <x:c r="Q27" s="11" t="str">
+        <x:v>Case-specific oracles: see test-matrix.csv, rows T18</x:v>
+      </x:c>
+      <x:c r="R27" s="11" t="str">
+        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
+      </x:c>
+      <x:c r="S27" s="11" t="str">
+        <x:v>Operational/quality acceptance pending</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70c3ba38ad99402a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83595676719f4c96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update M3 Person 2 evidence, RTM and PED handoff
</commit_message>
<xml_diff>
--- a/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
+++ b/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Person 2 RTM" sheetId="1" r:id="Rf43969e42baa4807"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Person 2 RTM" sheetId="1" r:id="R889ce99fadd84655"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34,7 +34,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -51,16 +51,6 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFC2E7F3"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFFFF"/>
-      </x:patternFill>
-    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -68,7 +58,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="11">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -94,12 +84,6 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -342,10 +326,6 @@
     <x:col min="13" max="13" width="46" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="34" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="40" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="62" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="62" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="62" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="62" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2">
@@ -409,18 +389,6 @@
       <x:c r="O6" s="8" t="str">
         <x:v>GitHub evidence</x:v>
       </x:c>
-      <x:c r="P6" s="8" t="str">
-        <x:v>M3 test cases</x:v>
-      </x:c>
-      <x:c r="Q6" s="8" t="str">
-        <x:v>M3 expected result</x:v>
-      </x:c>
-      <x:c r="R6" s="8" t="str">
-        <x:v>M3 actual evidence</x:v>
-      </x:c>
-      <x:c r="S6" s="8" t="str">
-        <x:v>M3 defects and acceptance status</x:v>
-      </x:c>
     </x:row>
     <x:row r="7" ht="95" customHeight="1">
       <x:c r="A7" s="4" t="str">
@@ -470,18 +438,6 @@
       <x:c r="O7" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P7" s="11" t="str">
-        <x:v>T23, M3-S01</x:v>
-      </x:c>
-      <x:c r="Q7" s="11" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T23, M3-S01</x:v>
-      </x:c>
-      <x:c r="R7" s="11" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S7" s="11" t="str">
-        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
-      </x:c>
     </x:row>
     <x:row r="8" ht="95" customHeight="1">
       <x:c r="A8" s="4" t="str">
@@ -531,18 +487,6 @@
       <x:c r="O8" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P8" s="12" t="str">
-        <x:v>T01, T02, T21, T23, M3-U01, M3-U02, M3-S01, M3-S02</x:v>
-      </x:c>
-      <x:c r="Q8" s="12" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T01, T02, T21, T23, M3-U01, M3-U02, M3-S01, M3-S02</x:v>
-      </x:c>
-      <x:c r="R8" s="12" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S8" s="12" t="str">
-        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
-      </x:c>
     </x:row>
     <x:row r="9" ht="95" customHeight="1">
       <x:c r="A9" s="4" t="str">
@@ -592,18 +536,6 @@
       <x:c r="O9" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P9" s="11" t="str">
-        <x:v>T02, T03</x:v>
-      </x:c>
-      <x:c r="Q9" s="11" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T02, T03</x:v>
-      </x:c>
-      <x:c r="R9" s="11" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S9" s="11" t="str">
-        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
-      </x:c>
     </x:row>
     <x:row r="10" ht="95" customHeight="1">
       <x:c r="A10" s="4" t="str">
@@ -653,18 +585,6 @@
       <x:c r="O10" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P10" s="12" t="str">
-        <x:v>T04, M3-S02</x:v>
-      </x:c>
-      <x:c r="Q10" s="12" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T04, M3-S02</x:v>
-      </x:c>
-      <x:c r="R10" s="12" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S10" s="12" t="str">
-        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
-      </x:c>
     </x:row>
     <x:row r="11" ht="95" customHeight="1">
       <x:c r="A11" s="4" t="str">
@@ -714,18 +634,6 @@
       <x:c r="O11" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P11" s="11" t="str">
-        <x:v>T09, M3-S01</x:v>
-      </x:c>
-      <x:c r="Q11" s="11" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T09, M3-S01</x:v>
-      </x:c>
-      <x:c r="R11" s="11" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S11" s="11" t="str">
-        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
-      </x:c>
     </x:row>
     <x:row r="12" ht="95" customHeight="1">
       <x:c r="A12" s="4" t="str">
@@ -775,18 +683,6 @@
       <x:c r="O12" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P12" s="12" t="str">
-        <x:v>T05, M3-S02</x:v>
-      </x:c>
-      <x:c r="Q12" s="12" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T05, M3-S02</x:v>
-      </x:c>
-      <x:c r="R12" s="12" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S12" s="12" t="str">
-        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
-      </x:c>
     </x:row>
     <x:row r="13" ht="95" customHeight="1">
       <x:c r="A13" s="4" t="str">
@@ -836,18 +732,6 @@
       <x:c r="O13" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P13" s="11" t="str">
-        <x:v>T14, T16</x:v>
-      </x:c>
-      <x:c r="Q13" s="11" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T14, T16</x:v>
-      </x:c>
-      <x:c r="R13" s="11" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S13" s="11" t="str">
-        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
-      </x:c>
     </x:row>
     <x:row r="14" ht="95" customHeight="1">
       <x:c r="A14" s="4" t="str">
@@ -866,7 +750,7 @@
       </x:c>
       <x:c r="E14" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">AC-F08: Assignment locks the ticket to one category-authorised owner. Ineligible owners or missing due dates abort the assignment. Reassignment preserves the prior owner in the history log and notifies the requester.</x:t>
+          <x:t>AC-F08: Assignment locks the ticket to one category-authorised owner. Ineligible owners or missing due dates abort the assignment. Reassignment preserves the prior owner in the history log and notifies the requester.</x:t>
         </x:is>
       </x:c>
       <x:c r="F14" s="4" t="str">
@@ -898,18 +782,6 @@
       </x:c>
       <x:c r="O14" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
-      </x:c>
-      <x:c r="P14" s="12" t="str">
-        <x:v>T06, T20, M3-S01</x:v>
-      </x:c>
-      <x:c r="Q14" s="12" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T06, T20, M3-S01</x:v>
-      </x:c>
-      <x:c r="R14" s="12" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S14" s="12" t="str">
-        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="95" customHeight="1">
@@ -960,18 +832,6 @@
       <x:c r="O15" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P15" s="11" t="str">
-        <x:v>T19, M3-U03, M3-U06</x:v>
-      </x:c>
-      <x:c r="Q15" s="11" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T19, M3-U03, M3-U06</x:v>
-      </x:c>
-      <x:c r="R15" s="11" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S15" s="11" t="str">
-        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
-      </x:c>
     </x:row>
     <x:row r="16" ht="95" customHeight="1">
       <x:c r="A16" s="4" t="str">
@@ -1021,18 +881,6 @@
       <x:c r="O16" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P16" s="12" t="str">
-        <x:v>T07, T08, M3-U05, M3-S01, M3-S02</x:v>
-      </x:c>
-      <x:c r="Q16" s="12" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T07, T08, M3-U05, M3-S01, M3-S02</x:v>
-      </x:c>
-      <x:c r="R16" s="12" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S16" s="12" t="str">
-        <x:v>DEF-M3-005; browser reasons pending</x:v>
-      </x:c>
     </x:row>
     <x:row r="17" ht="95" customHeight="1">
       <x:c r="A17" s="4" t="str">
@@ -1082,18 +930,6 @@
       <x:c r="O17" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P17" s="11" t="str">
-        <x:v>T09, T24, M3-S01</x:v>
-      </x:c>
-      <x:c r="Q17" s="11" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T09, T24, M3-S01</x:v>
-      </x:c>
-      <x:c r="R17" s="11" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S17" s="11" t="str">
-        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
-      </x:c>
     </x:row>
     <x:row r="18" ht="95" customHeight="1">
       <x:c r="A18" s="4" t="str">
@@ -1143,18 +979,6 @@
       <x:c r="O18" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P18" s="12" t="str">
-        <x:v>T13, T15, T16</x:v>
-      </x:c>
-      <x:c r="Q18" s="12" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T13, T15, T16</x:v>
-      </x:c>
-      <x:c r="R18" s="12" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S18" s="12" t="str">
-        <x:v>DEF-M3-004/006; browser acceptance pending</x:v>
-      </x:c>
     </x:row>
     <x:row r="19" ht="95" customHeight="1">
       <x:c r="A19" s="4" t="str">
@@ -1204,18 +1028,6 @@
       <x:c r="O19" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P19" s="11" t="str">
-        <x:v>T11, T12, T19, T20</x:v>
-      </x:c>
-      <x:c r="Q19" s="11" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T11, T12, T19, T20</x:v>
-      </x:c>
-      <x:c r="R19" s="11" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S19" s="11" t="str">
-        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
-      </x:c>
     </x:row>
     <x:row r="20" ht="95" customHeight="1">
       <x:c r="A20" s="4" t="str">
@@ -1240,7 +1052,7 @@
       </x:c>
       <x:c r="G20" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">users.role, requester_id and staff_categories authorisation</x:t>
+          <x:t>users.role, requester_id and staff_categories authorisation</x:t>
         </x:is>
       </x:c>
       <x:c r="H20" s="4" t="str">
@@ -1266,18 +1078,6 @@
       </x:c>
       <x:c r="O20" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
-      </x:c>
-      <x:c r="P20" s="12" t="str">
-        <x:v>T04, T05, T13, T22, T23, M3-I01</x:v>
-      </x:c>
-      <x:c r="Q20" s="12" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T04, T05, T13, T22, T23, M3-I01</x:v>
-      </x:c>
-      <x:c r="R20" s="12" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S20" s="12" t="str">
-        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="95" customHeight="1">
@@ -1306,7 +1106,7 @@
       </x:c>
       <x:c r="H21" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">HTTPS proposed; Secure cookie option; sanitised errors</x:t>
+          <x:t>HTTPS proposed; Secure cookie option; sanitised errors</x:t>
         </x:is>
       </x:c>
       <x:c r="I21" s="4" t="str">
@@ -1329,18 +1129,6 @@
       </x:c>
       <x:c r="O21" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
-      </x:c>
-      <x:c r="P21" s="11" t="str">
-        <x:v>T21, M3-I01, M3-I02</x:v>
-      </x:c>
-      <x:c r="Q21" s="11" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T21, M3-I01, M3-I02</x:v>
-      </x:c>
-      <x:c r="R21" s="11" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S21" s="11" t="str">
-        <x:v>DEF-M3-002 fixed locally; TLS/secret scan pending</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="95" customHeight="1">
@@ -1391,18 +1179,6 @@
       <x:c r="O22" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P22" s="12" t="str">
-        <x:v>T10, T11, T17, M3-U04, M3-S02</x:v>
-      </x:c>
-      <x:c r="Q22" s="12" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T10, T11, T17, M3-U04, M3-S02</x:v>
-      </x:c>
-      <x:c r="R22" s="12" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S22" s="12" t="str">
-        <x:v>Selected automated behaviour verified; full acceptance/approval separate</x:v>
-      </x:c>
     </x:row>
     <x:row r="23" ht="95" customHeight="1">
       <x:c r="A23" s="4" t="str">
@@ -1452,18 +1228,6 @@
       <x:c r="O23" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P23" s="11" t="str">
-        <x:v>No additional automated acceptance evidence</x:v>
-      </x:c>
-      <x:c r="Q23" s="11" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows No additional automated acceptance evidence</x:v>
-      </x:c>
-      <x:c r="R23" s="11" t="str">
-        <x:v>No qualifying local automation result</x:v>
-      </x:c>
-      <x:c r="S23" s="11" t="str">
-        <x:v>Operational/quality acceptance pending</x:v>
-      </x:c>
     </x:row>
     <x:row r="24" ht="95" customHeight="1">
       <x:c r="A24" s="4" t="str">
@@ -1512,18 +1276,6 @@
       </x:c>
       <x:c r="O24" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
-      </x:c>
-      <x:c r="P24" s="12" t="str">
-        <x:v>No additional automated acceptance evidence</x:v>
-      </x:c>
-      <x:c r="Q24" s="12" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows No additional automated acceptance evidence</x:v>
-      </x:c>
-      <x:c r="R24" s="12" t="str">
-        <x:v>No qualifying local automation result</x:v>
-      </x:c>
-      <x:c r="S24" s="12" t="str">
-        <x:v>Operational/quality acceptance pending</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="95" customHeight="1">
@@ -1575,18 +1327,6 @@
       <x:c r="O25" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P25" s="11" t="str">
-        <x:v>No additional automated acceptance evidence</x:v>
-      </x:c>
-      <x:c r="Q25" s="11" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows No additional automated acceptance evidence</x:v>
-      </x:c>
-      <x:c r="R25" s="11" t="str">
-        <x:v>No qualifying local automation result</x:v>
-      </x:c>
-      <x:c r="S25" s="11" t="str">
-        <x:v>Operational/quality acceptance pending</x:v>
-      </x:c>
     </x:row>
     <x:row r="26" ht="95" customHeight="1">
       <x:c r="A26" s="4" t="str">
@@ -1611,7 +1351,7 @@
       </x:c>
       <x:c r="G26" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Database health query; sanitised failure metadata</x:t>
+          <x:t>Database health query; sanitised failure metadata</x:t>
         </x:is>
       </x:c>
       <x:c r="H26" s="4" t="str">
@@ -1637,18 +1377,6 @@
       </x:c>
       <x:c r="O26" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
-      </x:c>
-      <x:c r="P26" s="12" t="str">
-        <x:v>M3-I03</x:v>
-      </x:c>
-      <x:c r="Q26" s="12" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows M3-I03</x:v>
-      </x:c>
-      <x:c r="R26" s="12" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S26" s="12" t="str">
-        <x:v>Operational/quality acceptance pending</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="95" customHeight="1">
@@ -1699,23 +1427,11 @@
       <x:c r="O27" s="10" t="str">
         <x:v>Pending actual issue/commit/PR/review; not fabricated</x:v>
       </x:c>
-      <x:c r="P27" s="11" t="str">
-        <x:v>T18</x:v>
-      </x:c>
-      <x:c r="Q27" s="11" t="str">
-        <x:v>Case-specific oracles: see test-matrix.csv, rows T18</x:v>
-      </x:c>
-      <x:c r="R27" s="11" t="str">
-        <x:v>after-fix.tap: named tests pass; browser/operational checks not inferred</x:v>
-      </x:c>
-      <x:c r="S27" s="11" t="str">
-        <x:v>Operational/quality acceptance pending</x:v>
-      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83595676719f4c96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70c3ba38ad99402a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct M4 acceptance scoring following PR review
</commit_message>
<xml_diff>
--- a/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
+++ b/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eduard Goosen\projects\CivicConnect\docs\milestone2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59912F4D-4991-4AB6-8574-53A2741B24BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C777B7B-7A60-4B6F-8DC5-5BE396323151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -919,33 +919,18 @@
     <t>T02/T03 verify active categories, rejection and preserved historical labels.</t>
   </si>
   <si>
-    <t>Own-record lists/status and isolation tested. Full requester detail/history functionality remains a requirement-level gap.</t>
-  </si>
-  <si>
     <t>Persisted public/internal activities exist; dashboard does not display the required explanations and summaries.</t>
   </si>
   <si>
     <t>Category isolation tested; staff details omit required fields/history.</t>
   </si>
   <si>
-    <t>API combined-filter/sort tests and empty-result UI exist; full browser search/filter controls remain a requirement-level gap.</t>
-  </si>
-  <si>
     <t>Owner eligibility, required due time and reassignment audit tested; requester-facing notification remains incomplete.</t>
   </si>
   <si>
     <t>Priority/date validation and audit tested; CR-P2-001 date-rule discrepancy remains unresolved.</t>
   </si>
   <si>
-    <t>Lifecycle and mandatory notes tested, including M4 browser journey; requester notification content remains incomplete.</t>
-  </si>
-  <si>
-    <t>API notes preserve metadata and explicit visibility; public projection and immutable history tested. Separate browser note controls remain absent.</t>
-  </si>
-  <si>
-    <t>API report calculations, date validation and oversight permissions tested. Oversight browser interface remains absent.</t>
-  </si>
-  <si>
     <t>Audit metadata, prior/new values, immutability and requester restrictions covered by existing tests.</t>
   </si>
   <si>
@@ -983,6 +968,21 @@
   </si>
   <si>
     <t>Provisional; team review pending; assessed 17 October 2026</t>
+  </si>
+  <si>
+    <t>Requester list/status and ownership isolation covered by existing tests. PR #29 adds details and public history; 17 October screenshots confirm submitted fields, receipt/assignment history and resolution feedback. Refresh/back passed. Separate final-candidate release verification remains pending.</t>
+  </si>
+  <si>
+    <t>API filtering/sorting tests pass, but complete staff browser search, combined filters and sorting controls are absent. API evidence alone does not establish the full staff workflow.</t>
+  </si>
+  <si>
+    <t>Automated lifecycle/mandatory-note cases pass. Resolution/rejection browser validation retains its 14 October date. Assumed M4 lifecycle passes were withdrawn. New requester history displays existing resolution feedback; full lifecycle notification acceptance remains incomplete.</t>
+  </si>
+  <si>
+    <t>API note metadata, explicit visibility and immutable history are tested. Requester public history and internal-note privacy were checked on 17 October. Separate staff browser note/visibility controls remain absent.</t>
+  </si>
+  <si>
+    <t>API report calculations, date validation and oversight permissions are tested. Oversight browser reporting is unavailable, so the complete user workflow is not accepted.</t>
   </si>
 </sst>
 </file>
@@ -1432,10 +1432,10 @@
         <v>283</v>
       </c>
       <c r="W6" s="6" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="X6" s="6" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="51">
@@ -1506,10 +1506,10 @@
         <v>284</v>
       </c>
       <c r="W7" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X7" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="63.75">
@@ -1580,10 +1580,10 @@
         <v>285</v>
       </c>
       <c r="W8" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X8" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="51">
@@ -1654,13 +1654,13 @@
         <v>286</v>
       </c>
       <c r="W9" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X9" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
-    <row r="10" spans="1:24" ht="51">
+    <row r="10" spans="1:24" ht="71.25">
       <c r="A10" s="2" t="s">
         <v>52</v>
       </c>
@@ -1725,13 +1725,13 @@
         <v>1</v>
       </c>
       <c r="V10" s="6" t="s">
-        <v>287</v>
+        <v>304</v>
       </c>
       <c r="W10" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X10" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="51">
@@ -1799,13 +1799,13 @@
         <v>0.5</v>
       </c>
       <c r="V11" s="6" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="W11" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X11" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="51">
@@ -1873,13 +1873,13 @@
         <v>0.5</v>
       </c>
       <c r="V12" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="W12" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X12" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="51">
@@ -1941,19 +1941,19 @@
         <v>265</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="U13" s="7">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V13" s="6" t="s">
-        <v>290</v>
+        <v>305</v>
       </c>
       <c r="W13" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X13" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="51">
@@ -2021,13 +2021,13 @@
         <v>0.5</v>
       </c>
       <c r="V14" s="6" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="W14" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X14" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="38.25">
@@ -2095,16 +2095,16 @@
         <v>0.5</v>
       </c>
       <c r="V15" s="6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="W15" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X15" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="51">
+    <row r="16" spans="1:24" ht="57">
       <c r="A16" s="2" t="s">
         <v>101</v>
       </c>
@@ -2169,13 +2169,13 @@
         <v>0.5</v>
       </c>
       <c r="V16" s="6" t="s">
-        <v>293</v>
+        <v>306</v>
       </c>
       <c r="W16" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X16" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="51">
@@ -2237,19 +2237,19 @@
         <v>271</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="U17" s="7">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V17" s="6" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="W17" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X17" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="18" spans="1:24" ht="51">
@@ -2311,19 +2311,19 @@
         <v>272</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="U18" s="7">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V18" s="6" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="W18" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X18" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="51">
@@ -2391,13 +2391,13 @@
         <v>1</v>
       </c>
       <c r="V19" s="6" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="W19" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X19" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="20" spans="1:24" ht="51">
@@ -2465,13 +2465,13 @@
         <v>1</v>
       </c>
       <c r="V20" s="6" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="W20" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X20" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="178.5">
@@ -2539,13 +2539,13 @@
         <v>0.5</v>
       </c>
       <c r="V21" s="6" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="W21" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X21" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="51">
@@ -2613,13 +2613,13 @@
         <v>0.5</v>
       </c>
       <c r="V22" s="6" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="W22" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X22" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="23" spans="1:24" ht="178.5">
@@ -2687,13 +2687,13 @@
         <v>0</v>
       </c>
       <c r="V23" s="6" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="W23" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X23" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="24" spans="1:24" ht="38.25">
@@ -2761,13 +2761,13 @@
         <v>0</v>
       </c>
       <c r="V24" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="W24" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="W24" s="6" t="s">
-        <v>306</v>
-      </c>
       <c r="X24" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="25" spans="1:24" ht="51">
@@ -2835,13 +2835,13 @@
         <v>0.5</v>
       </c>
       <c r="V25" s="6" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="W25" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X25" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="26" spans="1:24" ht="51">
@@ -2909,13 +2909,13 @@
         <v>0</v>
       </c>
       <c r="V26" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="W26" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="X26" s="6" t="s">
         <v>303</v>
-      </c>
-      <c r="W26" s="6" t="s">
-        <v>306</v>
-      </c>
-      <c r="X26" s="6" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="27" spans="1:24" ht="178.5">
@@ -2983,13 +2983,13 @@
         <v>0.5</v>
       </c>
       <c r="V27" s="6" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="W27" s="6" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="X27" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete M4 workflows and record measured acceptance evidence
</commit_message>
<xml_diff>
--- a/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
+++ b/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eduard Goosen\projects\CivicConnect\docs\milestone2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C777B7B-7A60-4B6F-8DC5-5BE396323151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C800577C-E089-4F24-AB73-376F96B8A698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="304">
   <si>
     <t>CivicConnect M2 Person 2 traceability</t>
   </si>
@@ -231,9 +231,6 @@
     <t>T01, T09, T19, T20</t>
   </si>
   <si>
-    <t>Backend activity feed implemented; UI highlights pending</t>
-  </si>
-  <si>
     <t>FR-006</t>
   </si>
   <si>
@@ -279,9 +276,6 @@
     <t>T14, T16</t>
   </si>
   <si>
-    <t>Implemented backend; in-memory filtering; load check pending</t>
-  </si>
-  <si>
     <t>ADR-P2-001; ADR-P2-002; ADR-P2-003; P2-R02</t>
   </si>
   <si>
@@ -304,9 +298,6 @@
     <t>T06, T10, T11, T20</t>
   </si>
   <si>
-    <t>Implemented candidate; due-date clarification pending</t>
-  </si>
-  <si>
     <t>ADR-P2-001; ADR-P2-002; ADR-P2-003; P2-R06; CR-P2-001</t>
   </si>
   <si>
@@ -412,9 +403,6 @@
     <t>T13, T15, T16</t>
   </si>
   <si>
-    <t>Implemented candidate; reporting interpretations pending</t>
-  </si>
-  <si>
     <t>ADR-P2-001; ADR-P2-002; ADR-P2-003; P2-R02; P2-R06</t>
   </si>
   <si>
@@ -519,9 +507,6 @@
   </si>
   <si>
     <t>T10, T11, T17; crash/multi-process tests Planned</t>
-  </si>
-  <si>
-    <t>Initial evidence only; semantic create deduplication undefined</t>
   </si>
   <si>
     <t>ADR-P2-001; ADR-P2-002; ADR-P2-003; P2-R01; P2-R02</t>
@@ -691,12 +676,6 @@
     <t>Partial: selected static/security and repository-hygiene checks have CI evidence; production TLS, network traffic audit, and comprehensive repository/build/log secret scanning remain unverified.</t>
   </si>
   <si>
-    <t>Partial performance evidence: configured smoke thresholds passed for the tested small workload. Formal AC-N04 workload (5,000 active records, 20 concurrent users, 15 minutes, 80/20 read-write mix) has not been run; no full NFR-004 compliance claim.</t>
-  </si>
-  <si>
-    <t>Partial: backup snapshot creation/readability and SQLite integrity are evidenced by the simulated staging CI flow. RTO &lt;=60 minutes, RPO &lt;=24 hours and off-site disaster recovery remain unproven.</t>
-  </si>
-  <si>
     <t>[PR #23 — CI, security, staging and performance implementation](https://github.com/Amelia-VanDerWalt/CivicConnect/pull/23); [PR #25 — merged Person 3 handoff](https://github.com/Amelia-VanDerWalt/CivicConnect/pull/25); [successful GitHub Actions run #30 on commit `98ff24f459de205cb125ab88a6c26e0ef5b27912`](https://github.com/Amelia-VanDerWalt/CivicConnect/actions/runs/38797557518); [PR #27 — PED/RTM integration and review](https://github.com/Amelia-VanDerWalt/CivicConnect/pull/27). The cited CI run is evidence for its recorded commit, not a substitute for a fresh run on the final submitted SHA.</t>
   </si>
   <si>
@@ -919,15 +898,6 @@
     <t>T02/T03 verify active categories, rejection and preserved historical labels.</t>
   </si>
   <si>
-    <t>Persisted public/internal activities exist; dashboard does not display the required explanations and summaries.</t>
-  </si>
-  <si>
-    <t>Category isolation tested; staff details omit required fields/history.</t>
-  </si>
-  <si>
-    <t>Owner eligibility, required due time and reassignment audit tested; requester-facing notification remains incomplete.</t>
-  </si>
-  <si>
     <t>Priority/date validation and audit tested; CR-P2-001 date-rule discrepancy remains unresolved.</t>
   </si>
   <si>
@@ -940,12 +910,6 @@
     <t>Selected repository hygiene checks exist; TLS and complete repository/log/build-output coverage are not established.</t>
   </si>
   <si>
-    <t>Rollback, stale edits and normal close/reopen persistence tested; forced-restart recovery not established.</t>
-  </si>
-  <si>
-    <t>Performance smoke evidence does not meet the specified workload and 15-minute test.</t>
-  </si>
-  <si>
     <t>Representative-user unassisted timed study not established.</t>
   </si>
   <si>
@@ -955,34 +919,55 @@
     <t>Timed outage alerts and required diagnostic-log properties not established.</t>
   </si>
   <si>
-    <t>Backup integrity/readback tested; timed full-system restoration not established.</t>
-  </si>
-  <si>
     <t>M4 assessed candidate</t>
   </si>
   <si>
-    <t>f52bb8fd6c15e4a72abf182a9b4fe43511f1027e</t>
-  </si>
-  <si>
     <t>M4 review status</t>
   </si>
   <si>
-    <t>Provisional; team review pending; assessed 17 October 2026</t>
-  </si>
-  <si>
     <t>Requester list/status and ownership isolation covered by existing tests. PR #29 adds details and public history; 17 October screenshots confirm submitted fields, receipt/assignment history and resolution feedback. Refresh/back passed. Separate final-candidate release verification remains pending.</t>
   </si>
   <si>
-    <t>API filtering/sorting tests pass, but complete staff browser search, combined filters and sorting controls are absent. API evidence alone does not establish the full staff workflow.</t>
-  </si>
-  <si>
-    <t>Automated lifecycle/mandatory-note cases pass. Resolution/rejection browser validation retains its 14 October date. Assumed M4 lifecycle passes were withdrawn. New requester history displays existing resolution feedback; full lifecycle notification acceptance remains incomplete.</t>
-  </si>
-  <si>
-    <t>API note metadata, explicit visibility and immutable history are tested. Requester public history and internal-note privacy were checked on 17 October. Separate staff browser note/visibility controls remain absent.</t>
-  </si>
-  <si>
-    <t>API report calculations, date validation and oversight permissions are tested. Oversight browser reporting is unavailable, so the complete user workflow is not accepted.</t>
+    <t>Implemented; selected automated and 18 October browser checks passed; peer review pending.</t>
+  </si>
+  <si>
+    <t>18 October: public notes, scheduling updates, resolution/closure feedback and requester sign-out persistence confirmed. Internal notes hidden. Existing automated activity/privacy cases pass.</t>
+  </si>
+  <si>
+    <t>18 October: staff queue/details show submitted fields, owner, priority, due date and history. Existing backend category/direct-access tests pass.</t>
+  </si>
+  <si>
+    <t>18 October: combined title/status filtering, no-results message and reset passed in the browser. Search/filter/sort controls implemented; existing automated combined-filter/null-last-sort cases pass.</t>
+  </si>
+  <si>
+    <t>18 October: Assigned to In progress to Resolved to Closed executed. Empty resolution summary blocked. Requester sees final status, summary and highlighted history. Existing rejection/transition tests pass; withdrawn 17 October assumptions remain withdrawn.</t>
+  </si>
+  <si>
+    <t>18 October: explicit Public/Internal browser note controls saved notes; public note visible to requester and Internal note hidden. Staff history displays metadata/visibility. Existing immutable-history cases pass.</t>
+  </si>
+  <si>
+    <t>18 October: Oversight report screen, date filtering, empty results and read-only details passed. Existing automated report/date/MTTR/role cases pass; browser observations do not independently recompute every metric.</t>
+  </si>
+  <si>
+    <t>Implemented; measured M4 checks passed in the recorded local environment; peer review pending.</t>
+  </si>
+  <si>
+    <t>Assignment and reassignment controls implemented. Isolated automated check changed eligible owner 3 to 5, verified prior/new audit values and requester-visible feedback, and rejected ineligible/missing-date assignments without mutation. Browser controls were inspected; this reassignment execution was API-based.</t>
+  </si>
+  <si>
+    <t>Forced application termination preserved all acknowledged requests, activities, accounts and category permissions. Integrity checks passed. Existing rollback/stale-edit cases and the additional conflict check passed. Process-crash evidence does not establish host power-loss behaviour.</t>
+  </si>
+  <si>
+    <t>Formal local workload passed: 900.015 seconds, 5000 initial active records, 20 concurrent virtual users, 7200 reads and 1800 writes. Read p95 395.5 ms; write p95 42.86 ms. Response content and acknowledged-write persistence checked. Loopback HTTP environment; not a production network claim.</t>
+  </si>
+  <si>
+    <t>Local backup restoration drill passed in 1262.77 ms. Restored server health, account access, requests, activities, permissions and report counts verified; zero acknowledged business-record loss in this drill. Fresh same-host snapshot; ongoing backup schedule, off-site retention and disaster-site recovery remain unproven.</t>
+  </si>
+  <si>
+    <t>11dc19df95590aa9daf518e0f04441cf389ad0ed plus runtime files fingerprinted in m4-formal-load-results.json</t>
+  </si>
+  <si>
+    <t>Provisional 18 October 2026; team review and final release approval pending</t>
   </si>
 </sst>
 </file>
@@ -1411,34 +1396,34 @@
         <v>17</v>
       </c>
       <c r="P6" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="Q6" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="R6" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="S6" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="U6" s="6" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="V6" s="6" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="W6" s="6" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="X6" s="6" t="s">
-        <v>302</v>
+        <v>288</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="51">
+    <row r="7" spans="1:24" ht="57">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -1485,28 +1470,28 @@
         <v>32</v>
       </c>
       <c r="P7" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="Q7" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="R7" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="S7" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="U7" s="7">
         <v>1</v>
       </c>
       <c r="V7" s="6" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="W7" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X7" s="6" t="s">
         <v>303</v>
@@ -1559,34 +1544,34 @@
         <v>32</v>
       </c>
       <c r="P8" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="Q8" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="R8" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="S8" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="U8" s="7">
         <v>1</v>
       </c>
       <c r="V8" s="6" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="W8" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X8" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="9" spans="1:24" ht="51">
+    <row r="9" spans="1:24" ht="57">
       <c r="A9" s="2" t="s">
         <v>43</v>
       </c>
@@ -1636,25 +1621,25 @@
         <v>50</v>
       </c>
       <c r="Q9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="R9" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="S9" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="U9" s="7">
         <v>1</v>
       </c>
       <c r="V9" s="6" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="W9" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X9" s="6" t="s">
         <v>303</v>
@@ -1707,34 +1692,34 @@
         <v>32</v>
       </c>
       <c r="P10" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="Q10" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="R10" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="S10" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="T10" s="6" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="U10" s="7">
         <v>1</v>
       </c>
       <c r="V10" s="6" t="s">
-        <v>304</v>
+        <v>289</v>
       </c>
       <c r="W10" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X10" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="51">
+    <row r="11" spans="1:24" ht="57">
       <c r="A11" s="2" t="s">
         <v>60</v>
       </c>
@@ -1769,7 +1754,7 @@
         <v>66</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>67</v>
+        <v>290</v>
       </c>
       <c r="M11" s="2" t="s">
         <v>30</v>
@@ -1781,54 +1766,54 @@
         <v>32</v>
       </c>
       <c r="P11" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="Q11" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="R11" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="S11" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="T11" s="6" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="U11" s="7">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V11" s="6" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="W11" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X11" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="12" spans="1:24" ht="51">
+    <row r="12" spans="1:24" ht="57">
       <c r="A12" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>56</v>
@@ -1837,13 +1822,13 @@
         <v>26</v>
       </c>
       <c r="J12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="K12" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="K12" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="L12" s="2" t="s">
-        <v>59</v>
+        <v>290</v>
       </c>
       <c r="M12" s="2" t="s">
         <v>30</v>
@@ -1855,72 +1840,72 @@
         <v>32</v>
       </c>
       <c r="P12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="Q12" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="R12" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="S12" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="U12" s="7">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V12" s="6" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="W12" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X12" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="51">
+    <row r="13" spans="1:24" ht="57">
       <c r="A13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="C13" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G13" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J13" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="K13" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="L13" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="M13" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>83</v>
       </c>
       <c r="N13" s="5" t="s">
         <v>31</v>
@@ -1929,72 +1914,72 @@
         <v>32</v>
       </c>
       <c r="P13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q13" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="R13" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="S13" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="U13" s="7">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V13" s="6" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="W13" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X13" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="14" spans="1:24" ht="51">
+    <row r="14" spans="1:24" ht="71.25">
       <c r="A14" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J14" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="M14" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="N14" s="5" t="s">
         <v>31</v>
@@ -2003,72 +1988,72 @@
         <v>32</v>
       </c>
       <c r="P14" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="Q14" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="R14" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="S14" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="U14" s="7">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V14" s="6" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="W14" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X14" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="15" spans="1:24" ht="38.25">
+    <row r="15" spans="1:24" ht="57">
       <c r="A15" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="N15" s="5" t="s">
         <v>31</v>
@@ -2077,28 +2062,28 @@
         <v>32</v>
       </c>
       <c r="P15" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="Q15" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="R15" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="S15" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="U15" s="7">
         <v>0.5</v>
       </c>
       <c r="V15" s="6" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="W15" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X15" s="6" t="s">
         <v>303</v>
@@ -2106,40 +2091,40 @@
     </row>
     <row r="16" spans="1:24" ht="57">
       <c r="A16" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>29</v>
+        <v>290</v>
       </c>
       <c r="M16" s="2" t="s">
         <v>42</v>
@@ -2151,72 +2136,72 @@
         <v>32</v>
       </c>
       <c r="P16" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="Q16" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="R16" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="S16" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="T16" s="6" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="U16" s="7">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V16" s="6" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="W16" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X16" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="17" spans="1:24" ht="51">
+    <row r="17" spans="1:24" ht="57">
       <c r="A17" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>59</v>
+        <v>290</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="N17" s="5" t="s">
         <v>31</v>
@@ -2225,72 +2210,72 @@
         <v>32</v>
       </c>
       <c r="P17" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="Q17" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="R17" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="S17" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="U17" s="7">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V17" s="6" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="W17" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X17" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="18" spans="1:24" ht="51">
+    <row r="18" spans="1:24" ht="57">
       <c r="A18" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>124</v>
+        <v>290</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="N18" s="5" t="s">
         <v>31</v>
@@ -2299,72 +2284,72 @@
         <v>32</v>
       </c>
       <c r="P18" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="Q18" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="R18" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="S18" t="s">
+        <v>265</v>
+      </c>
+      <c r="T18" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="T18" s="6" t="s">
-        <v>280</v>
-      </c>
       <c r="U18" s="7">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V18" s="6" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="W18" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X18" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="19" spans="1:24" ht="51">
+    <row r="19" spans="1:24" ht="57">
       <c r="A19" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="N19" s="5" t="s">
         <v>31</v>
@@ -2373,69 +2358,69 @@
         <v>32</v>
       </c>
       <c r="P19" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="Q19" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="R19" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="S19" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="U19" s="7">
         <v>1</v>
       </c>
       <c r="V19" s="6" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
       <c r="W19" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X19" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="20" spans="1:24" ht="51">
+    <row r="20" spans="1:24" ht="57">
       <c r="A20" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="M20" s="2" t="s">
         <v>30</v>
@@ -2447,28 +2432,28 @@
         <v>32</v>
       </c>
       <c r="P20" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="Q20" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="R20" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="S20" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="U20" s="7">
         <v>1</v>
       </c>
       <c r="V20" s="6" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="W20" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X20" s="6" t="s">
         <v>303</v>
@@ -2476,117 +2461,117 @@
     </row>
     <row r="21" spans="1:24" ht="178.5">
       <c r="A21" s="2" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="N21" s="5" t="s">
         <v>31</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="P21" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="Q21" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="R21" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="S21" t="s">
+        <v>266</v>
+      </c>
+      <c r="T21" s="6" t="s">
         <v>273</v>
-      </c>
-      <c r="T21" s="6" t="s">
-        <v>280</v>
       </c>
       <c r="U21" s="7">
         <v>0.5</v>
       </c>
       <c r="V21" s="6" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="W21" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X21" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="22" spans="1:24" ht="51">
+    <row r="22" spans="1:24" ht="57">
       <c r="A22" s="2" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>158</v>
+        <v>297</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="N22" s="5" t="s">
         <v>31</v>
@@ -2595,28 +2580,28 @@
         <v>32</v>
       </c>
       <c r="P22" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="Q22" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="R22" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="S22" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="T22" s="6" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="U22" s="7">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V22" s="6" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="W22" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X22" s="6" t="s">
         <v>303</v>
@@ -2624,114 +2609,114 @@
     </row>
     <row r="23" spans="1:24" ht="178.5">
       <c r="A23" s="2" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>211</v>
+        <v>297</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="N23" s="5" t="s">
         <v>31</v>
       </c>
       <c r="O23" s="5" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="P23" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="Q23" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="R23" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="S23" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="T23" s="6" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="U23" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V23" s="6" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="W23" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X23" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="24" spans="1:24" ht="38.25">
+    <row r="24" spans="1:24" ht="57">
       <c r="A24" s="2" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="M24" s="2" t="s">
         <v>42</v>
@@ -2743,69 +2728,69 @@
         <v>32</v>
       </c>
       <c r="P24" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="Q24" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="R24" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="S24" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="T24" s="6" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="U24" s="7">
         <v>0</v>
       </c>
       <c r="V24" s="6" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
       <c r="W24" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X24" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="51">
+    <row r="25" spans="1:24" ht="57">
       <c r="A25" s="2" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="M25" s="2" t="s">
         <v>42</v>
@@ -2817,72 +2802,72 @@
         <v>32</v>
       </c>
       <c r="P25" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="Q25" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="R25" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="S25" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="T25" s="6" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="U25" s="7">
         <v>0.5</v>
       </c>
       <c r="V25" s="6" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
       <c r="W25" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X25" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="26" spans="1:24" ht="51">
+    <row r="26" spans="1:24" ht="57">
       <c r="A26" s="2" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="N26" s="5" t="s">
         <v>31</v>
@@ -2891,28 +2876,28 @@
         <v>32</v>
       </c>
       <c r="P26" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="Q26" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="R26" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="S26" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="T26" s="6" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="U26" s="7">
         <v>0</v>
       </c>
       <c r="V26" s="6" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
       <c r="W26" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X26" s="6" t="s">
         <v>303</v>
@@ -2920,73 +2905,73 @@
     </row>
     <row r="27" spans="1:24" ht="178.5">
       <c r="A27" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>212</v>
+        <v>297</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="N27" s="5" t="s">
         <v>31</v>
       </c>
       <c r="O27" s="5" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="P27" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="Q27" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="R27" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="S27" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="T27" s="6" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="U27" s="7">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V27" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="W27" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="X27" s="6" t="s">
         <v>303</v>

</xml_diff>

<commit_message>
Record approved M4 decisions and reconcile final acceptance
</commit_message>
<xml_diff>
--- a/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
+++ b/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eduard Goosen\projects\CivicConnect\docs\milestone2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C800577C-E089-4F24-AB73-376F96B8A698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7FBB62A-1F9F-4C25-9BD2-F394597C0F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="307">
   <si>
     <t>CivicConnect M2 Person 2 traceability</t>
   </si>
@@ -325,9 +325,6 @@
   </si>
   <si>
     <t>T19</t>
-  </si>
-  <si>
-    <t>Implemented candidate; rule and UI acceptance pending</t>
   </si>
   <si>
     <t>FR-010</t>
@@ -898,9 +895,6 @@
     <t>T02/T03 verify active categories, rejection and preserved historical labels.</t>
   </si>
   <si>
-    <t>Priority/date validation and audit tested; CR-P2-001 date-rule discrepancy remains unresolved.</t>
-  </si>
-  <si>
     <t>Audit metadata, prior/new values, immutability and requester restrictions covered by existing tests.</t>
   </si>
   <si>
@@ -968,6 +962,21 @@
   </si>
   <si>
     <t>Provisional 18 October 2026; team review and final release approval pending</t>
+  </si>
+  <si>
+    <t>Implemented; scheduling browser check and automated validation/audit evidence recorded.</t>
+  </si>
+  <si>
+    <t>CR-P2-001 approved by Edward, Albert and Amelia on 18 October 2026; see PR #28 discussion. Final release approval remains separate.</t>
+  </si>
+  <si>
+    <t>https://github.com/Amelia-VanDerWalt/CivicConnect/pull/28</t>
+  </si>
+  <si>
+    <t>AC-F09 supported by T19, M3-U03 and M3-U06, plus the recorded 18 October browser scheduling check. Valid priorities/future dates save; invalid values are rejected; audit retains previous values, actor, timestamp and reason. CR-P2-001 approved in PR #28: due dates must be strictly later than server current time when assigned or rescheduled.</t>
+  </si>
+  <si>
+    <t>FR-009 reassessed after recorded team clarification approval, 18 October 2026; final release approval remains separate.</t>
   </si>
 </sst>
 </file>
@@ -1396,31 +1405,31 @@
         <v>17</v>
       </c>
       <c r="P6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="Q6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="R6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S6" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U6" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="V6" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="V6" s="6" t="s">
-        <v>276</v>
-      </c>
       <c r="W6" s="6" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="X6" s="6" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="57">
@@ -1470,31 +1479,31 @@
         <v>32</v>
       </c>
       <c r="P7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U7" s="7">
         <v>1</v>
       </c>
       <c r="V7" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="W7" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X7" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="63.75">
@@ -1544,31 +1553,31 @@
         <v>32</v>
       </c>
       <c r="P8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Q8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="R8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="S8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U8" s="7">
         <v>1</v>
       </c>
       <c r="V8" s="6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="W8" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X8" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="57">
@@ -1621,28 +1630,28 @@
         <v>50</v>
       </c>
       <c r="Q9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="R9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U9" s="7">
         <v>1</v>
       </c>
       <c r="V9" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="W9" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X9" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="10" spans="1:24" ht="71.25">
@@ -1692,31 +1701,31 @@
         <v>32</v>
       </c>
       <c r="P10" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="Q10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="R10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="S10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="T10" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U10" s="7">
         <v>1</v>
       </c>
       <c r="V10" s="6" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="W10" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X10" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="57">
@@ -1754,7 +1763,7 @@
         <v>66</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="M11" s="2" t="s">
         <v>30</v>
@@ -1766,31 +1775,31 @@
         <v>32</v>
       </c>
       <c r="P11" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="Q11" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="R11" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S11" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="T11" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U11" s="7">
         <v>1</v>
       </c>
       <c r="V11" s="6" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="W11" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X11" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="57">
@@ -1828,7 +1837,7 @@
         <v>73</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="M12" s="2" t="s">
         <v>30</v>
@@ -1840,31 +1849,31 @@
         <v>32</v>
       </c>
       <c r="P12" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="Q12" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="R12" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="S12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U12" s="7">
         <v>1</v>
       </c>
       <c r="V12" s="6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="W12" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X12" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="57">
@@ -1902,7 +1911,7 @@
         <v>80</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="M13" s="2" t="s">
         <v>81</v>
@@ -1917,28 +1926,28 @@
         <v>80</v>
       </c>
       <c r="Q13" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="R13" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S13" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U13" s="7">
         <v>1</v>
       </c>
       <c r="V13" s="6" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="W13" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X13" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="71.25">
@@ -1955,7 +1964,7 @@
         <v>21</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>23</v>
@@ -1976,7 +1985,7 @@
         <v>87</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="M14" s="2" t="s">
         <v>88</v>
@@ -1988,34 +1997,34 @@
         <v>32</v>
       </c>
       <c r="P14" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="Q14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="R14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="S14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U14" s="7">
         <v>1</v>
       </c>
       <c r="V14" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="W14" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X14" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
-    <row r="15" spans="1:24" ht="57">
+    <row r="15" spans="1:24" ht="71.25">
       <c r="A15" s="2" t="s">
         <v>89</v>
       </c>
@@ -2050,51 +2059,51 @@
         <v>96</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>97</v>
+        <v>302</v>
       </c>
       <c r="M15" s="2" t="s">
         <v>88</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>31</v>
+        <v>303</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>32</v>
+        <v>304</v>
       </c>
       <c r="P15" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="Q15" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="R15" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S15" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="U15" s="7">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V15" s="6" t="s">
-        <v>280</v>
+        <v>305</v>
       </c>
       <c r="W15" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X15" s="6" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="16" spans="1:24" ht="57">
       <c r="A16" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>69</v>
@@ -2103,28 +2112,28 @@
         <v>21</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G16" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J16" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K16" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="L16" s="2" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="M16" s="2" t="s">
         <v>42</v>
@@ -2136,39 +2145,39 @@
         <v>32</v>
       </c>
       <c r="P16" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="Q16" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="R16" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="S16" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="T16" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U16" s="7">
         <v>1</v>
       </c>
       <c r="V16" s="6" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="W16" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X16" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="57">
       <c r="A17" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>106</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>69</v>
@@ -2177,31 +2186,31 @@
         <v>21</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G17" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J17" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="K17" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="L17" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="M17" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="N17" s="5" t="s">
         <v>31</v>
@@ -2210,72 +2219,72 @@
         <v>32</v>
       </c>
       <c r="P17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Q17" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R17" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S17" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U17" s="7">
         <v>1</v>
       </c>
       <c r="V17" s="6" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="W17" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X17" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="18" spans="1:24" ht="57">
       <c r="A18" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G18" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H18" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J18" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="K18" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="K18" s="2" t="s">
+      <c r="L18" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="M18" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="N18" s="5" t="s">
         <v>31</v>
@@ -2284,39 +2293,39 @@
         <v>32</v>
       </c>
       <c r="P18" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Q18" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="R18" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S18" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U18" s="7">
         <v>1</v>
       </c>
       <c r="V18" s="6" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="W18" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X18" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="57">
       <c r="A19" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>91</v>
@@ -2325,31 +2334,31 @@
         <v>21</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G19" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H19" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J19" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="K19" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="L19" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="L19" s="2" t="s">
+      <c r="M19" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>130</v>
       </c>
       <c r="N19" s="5" t="s">
         <v>31</v>
@@ -2358,69 +2367,69 @@
         <v>32</v>
       </c>
       <c r="P19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q19" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="R19" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S19" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U19" s="7">
         <v>1</v>
       </c>
       <c r="V19" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="W19" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X19" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="20" spans="1:24" ht="57">
       <c r="A20" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J20" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="K20" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="K20" s="2" t="s">
+      <c r="L20" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>138</v>
       </c>
       <c r="M20" s="2" t="s">
         <v>30</v>
@@ -2432,146 +2441,146 @@
         <v>32</v>
       </c>
       <c r="P20" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="Q20" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="R20" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S20" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U20" s="7">
         <v>1</v>
       </c>
       <c r="V20" s="6" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="W20" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X20" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="178.5">
       <c r="A21" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J21" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="M21" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>145</v>
       </c>
       <c r="N21" s="5" t="s">
         <v>31</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P21" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="Q21" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="R21" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="S21" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="T21" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="U21" s="7">
         <v>0.5</v>
       </c>
       <c r="V21" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="W21" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X21" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="57">
       <c r="A22" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G22" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>151</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J22" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="K22" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="K22" s="2" t="s">
+      <c r="L22" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="M22" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="L22" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>154</v>
       </c>
       <c r="N22" s="5" t="s">
         <v>31</v>
@@ -2580,69 +2589,69 @@
         <v>32</v>
       </c>
       <c r="P22" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="Q22" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="R22" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S22" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="T22" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U22" s="7">
         <v>1</v>
       </c>
       <c r="V22" s="6" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="W22" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X22" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="23" spans="1:24" ht="178.5">
       <c r="A23" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="E23" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G23" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="H23" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>161</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="M23" s="2" t="s">
         <v>81</v>
@@ -2651,72 +2660,72 @@
         <v>31</v>
       </c>
       <c r="O23" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P23" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="Q23" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="R23" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="S23" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="T23" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U23" s="7">
         <v>1</v>
       </c>
       <c r="V23" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="W23" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="W23" s="6" t="s">
-        <v>302</v>
-      </c>
       <c r="X23" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="24" spans="1:24" ht="57">
       <c r="A24" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G24" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H24" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J24" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="K24" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="K24" s="2" t="s">
+      <c r="L24" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>170</v>
       </c>
       <c r="M24" s="2" t="s">
         <v>42</v>
@@ -2728,69 +2737,69 @@
         <v>32</v>
       </c>
       <c r="P24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="Q24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="R24" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="S24" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T24" s="6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="U24" s="7">
         <v>0</v>
       </c>
       <c r="V24" s="6" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="W24" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X24" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="25" spans="1:24" ht="57">
       <c r="A25" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="D25" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>174</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G25" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="H25" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>176</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J25" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="K25" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="K25" s="2" t="s">
+      <c r="L25" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="M25" s="2" t="s">
         <v>42</v>
@@ -2802,72 +2811,72 @@
         <v>32</v>
       </c>
       <c r="P25" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="Q25" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="R25" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="S25" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="T25" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="U25" s="7">
         <v>0.5</v>
       </c>
       <c r="V25" s="6" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="W25" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X25" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="26" spans="1:24" ht="57">
       <c r="A26" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>181</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>182</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J26" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="K26" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="K26" s="2" t="s">
+      <c r="L26" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="L26" s="2" t="s">
+      <c r="M26" s="2" t="s">
         <v>187</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>188</v>
       </c>
       <c r="N26" s="5" t="s">
         <v>31</v>
@@ -2876,105 +2885,105 @@
         <v>32</v>
       </c>
       <c r="P26" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="Q26" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="R26" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S26" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T26" s="6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="U26" s="7">
         <v>0</v>
       </c>
       <c r="V26" s="6" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="W26" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="X26" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="27" spans="1:24" ht="178.5">
       <c r="A27" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>190</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>191</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G27" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>194</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>26</v>
       </c>
       <c r="J27" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="M27" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>196</v>
       </c>
       <c r="N27" s="5" t="s">
         <v>31</v>
       </c>
       <c r="O27" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="Q27" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="R27" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="S27" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="T27" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U27" s="7">
         <v>1</v>
       </c>
       <c r="V27" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="W27" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="X27" s="6" t="s">
         <v>301</v>
-      </c>
-      <c r="W27" s="6" t="s">
-        <v>302</v>
-      </c>
-      <c r="X27" s="6" t="s">
-        <v>303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Synchronise Excel RTM with reconciled JSON
</commit_message>
<xml_diff>
--- a/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
+++ b/docs/milestone2/CivicConnect_Milestone2_Person2_RTM_SA_English.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eduard Goosen\projects\CivicConnect\docs\milestone2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7FBB62A-1F9F-4C25-9BD2-F394597C0F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460894DF-FBB0-41FC-AF2E-42BB1C5BAD36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="306">
   <si>
     <t>CivicConnect M2 Person 2 traceability</t>
   </si>
@@ -754,9 +754,6 @@
     <t>Invalid assignment rejected; valid assignment version 2; New owner saved; old owner retained in audit; 201 create;200 valid changes;Closed visible;internal note hidden;logout denies read</t>
   </si>
   <si>
-    <t>Before/after actor and reason recorded; Only Low Normal High accepted; Only future timezone-bearing due accepted;CR-P2-001 pending</t>
-  </si>
-  <si>
     <t>Valid order succeeds; invalid transitions rejected; Reason required; rejected record terminal; Only valid transitions with required reason accepted; 201 create;200 valid changes;Closed visible;internal note hidden;logout denies read; 400 invalid;404 isolated reads;reason required;Rejected public reason;409 stale without extra activity</t>
   </si>
   <si>
@@ -958,12 +955,6 @@
     <t>Local backup restoration drill passed in 1262.77 ms. Restored server health, account access, requests, activities, permissions and report counts verified; zero acknowledged business-record loss in this drill. Fresh same-host snapshot; ongoing backup schedule, off-site retention and disaster-site recovery remain unproven.</t>
   </si>
   <si>
-    <t>11dc19df95590aa9daf518e0f04441cf389ad0ed plus runtime files fingerprinted in m4-formal-load-results.json</t>
-  </si>
-  <si>
-    <t>Provisional 18 October 2026; team review and final release approval pending</t>
-  </si>
-  <si>
     <t>Implemented; scheduling browser check and automated validation/audit evidence recorded.</t>
   </si>
   <si>
@@ -976,7 +967,13 @@
     <t>AC-F09 supported by T19, M3-U03 and M3-U06, plus the recorded 18 October browser scheduling check. Valid priorities/future dates save; invalid values are rejected; audit retains previous values, actor, timestamp and reason. CR-P2-001 approved in PR #28: due dates must be strictly later than server current time when assigned or rescheduled.</t>
   </si>
   <si>
-    <t>FR-009 reassessed after recorded team clarification approval, 18 October 2026; final release approval remains separate.</t>
+    <t>Integrated assessment baseline: 5d6069822d4c125ce642a5d119a28ca4555a2b32. Release owner reports hosted CI #88 SUCCESS on this candidate. Original local test provenance: 11dc19df95590aa9daf518e0f04441cf389ad0ed plus runtime files fingerprinted in m4-formal-load-results.json</t>
+  </si>
+  <si>
+    <t>Assessment reconciled through merged PR #34 on 18 October 2026. CR-P2-001 approved and DEF-M3-006 closed through team confirmations in PR #28. Remaining Partial/Not Met results are retained. Production release is not approved; submission SHA and matching CI must be confirmed after the final documentation merge.</t>
+  </si>
+  <si>
+    <t>Before/after values, actor, timestamp and reason recorded; only Low, Normal and High accepted; only future timezone-bearing due dates accepted. Historical M3 expectation: CR-P2-001 was pending at that time. Current decision: approved by the team on 18 October 2026; see PR #28.</t>
   </si>
 </sst>
 </file>
@@ -1064,7 +1061,6 @@
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <numFmt numFmtId="164" formatCode="0\.0"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1074,6 +1070,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="0\.0"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1114,11 +1111,11 @@
     <tableColumn id="17" xr3:uid="{1917B32C-7827-4253-A6A8-F9C5E18F4B3E}" name="M3 expected result"/>
     <tableColumn id="18" xr3:uid="{EC003B03-19AD-4350-9010-F806E7229BB0}" name="M3 actual evidence"/>
     <tableColumn id="19" xr3:uid="{9FCF144F-18DB-429D-A649-B317019406FF}" name="M3 defects and acceptance status"/>
-    <tableColumn id="20" xr3:uid="{D33923B3-C238-4FB2-BF1E-EE94CBF5C3DD}" name="M4 acceptance assessment" dataDxfId="2"/>
-    <tableColumn id="21" xr3:uid="{1F4CFEE8-123A-446D-9F53-B19A758C07CE}" name="M4 acceptance score" dataDxfId="0"/>
-    <tableColumn id="22" xr3:uid="{87A73715-9CB2-4A43-B3A9-9A7FCCAE7AB1}" name="M4 evidence and remaining gaps" dataDxfId="1"/>
-    <tableColumn id="23" xr3:uid="{F36858C7-60C5-4308-84A2-18F24A1F3D07}" name="M4 assessed candidate" dataDxfId="4"/>
-    <tableColumn id="24" xr3:uid="{5BDEFEFA-D79C-41AA-BDCA-020DC1DF5AAE}" name="M4 review status" dataDxfId="3"/>
+    <tableColumn id="20" xr3:uid="{D33923B3-C238-4FB2-BF1E-EE94CBF5C3DD}" name="M4 acceptance assessment" dataDxfId="4"/>
+    <tableColumn id="21" xr3:uid="{1F4CFEE8-123A-446D-9F53-B19A758C07CE}" name="M4 acceptance score" dataDxfId="3"/>
+    <tableColumn id="22" xr3:uid="{87A73715-9CB2-4A43-B3A9-9A7FCCAE7AB1}" name="M4 evidence and remaining gaps" dataDxfId="2"/>
+    <tableColumn id="23" xr3:uid="{F36858C7-60C5-4308-84A2-18F24A1F3D07}" name="M4 assessed candidate" dataDxfId="1"/>
+    <tableColumn id="24" xr3:uid="{5BDEFEFA-D79C-41AA-BDCA-020DC1DF5AAE}" name="M4 review status" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1358,7 +1355,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:24" ht="45">
+    <row r="6" spans="1:24" ht="42.75">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1411,28 +1408,28 @@
         <v>223</v>
       </c>
       <c r="R6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="S6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="U6" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="V6" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="V6" s="6" t="s">
-        <v>275</v>
-      </c>
       <c r="W6" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="X6" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="X6" s="6" t="s">
-        <v>286</v>
-      </c>
     </row>
-    <row r="7" spans="1:24" ht="57">
+    <row r="7" spans="1:24" ht="142.5">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -1485,28 +1482,28 @@
         <v>224</v>
       </c>
       <c r="R7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U7" s="7">
         <v>1</v>
       </c>
       <c r="V7" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="W7" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X7" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="63.75">
+    <row r="8" spans="1:24" ht="142.5">
       <c r="A8" s="2" t="s">
         <v>33</v>
       </c>
@@ -1559,28 +1556,28 @@
         <v>225</v>
       </c>
       <c r="R8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="S8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U8" s="7">
         <v>1</v>
       </c>
       <c r="V8" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="W8" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X8" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="9" spans="1:24" ht="57">
+    <row r="9" spans="1:24" ht="142.5">
       <c r="A9" s="2" t="s">
         <v>43</v>
       </c>
@@ -1633,28 +1630,28 @@
         <v>226</v>
       </c>
       <c r="R9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U9" s="7">
         <v>1</v>
       </c>
       <c r="V9" s="6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="W9" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X9" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="10" spans="1:24" ht="71.25">
+    <row r="10" spans="1:24" ht="142.5">
       <c r="A10" s="2" t="s">
         <v>52</v>
       </c>
@@ -1707,28 +1704,28 @@
         <v>227</v>
       </c>
       <c r="R10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="S10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="T10" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U10" s="7">
         <v>1</v>
       </c>
       <c r="V10" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="W10" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X10" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="57">
+    <row r="11" spans="1:24" ht="142.5">
       <c r="A11" s="2" t="s">
         <v>60</v>
       </c>
@@ -1763,7 +1760,7 @@
         <v>66</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="M11" s="2" t="s">
         <v>30</v>
@@ -1781,28 +1778,28 @@
         <v>228</v>
       </c>
       <c r="R11" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="T11" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U11" s="7">
         <v>1</v>
       </c>
       <c r="V11" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="W11" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X11" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="12" spans="1:24" ht="57">
+    <row r="12" spans="1:24" ht="142.5">
       <c r="A12" s="2" t="s">
         <v>67</v>
       </c>
@@ -1837,7 +1834,7 @@
         <v>73</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="M12" s="2" t="s">
         <v>30</v>
@@ -1855,28 +1852,28 @@
         <v>229</v>
       </c>
       <c r="R12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="S12" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U12" s="7">
         <v>1</v>
       </c>
       <c r="V12" s="6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="W12" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X12" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="57">
+    <row r="13" spans="1:24" ht="142.5">
       <c r="A13" s="2" t="s">
         <v>74</v>
       </c>
@@ -1911,7 +1908,7 @@
         <v>80</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="M13" s="2" t="s">
         <v>81</v>
@@ -1929,28 +1926,28 @@
         <v>230</v>
       </c>
       <c r="R13" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S13" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U13" s="7">
         <v>1</v>
       </c>
       <c r="V13" s="6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="W13" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X13" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="14" spans="1:24" ht="71.25">
+    <row r="14" spans="1:24" ht="142.5">
       <c r="A14" s="2" t="s">
         <v>82</v>
       </c>
@@ -1985,7 +1982,7 @@
         <v>87</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="M14" s="2" t="s">
         <v>88</v>
@@ -2003,28 +2000,28 @@
         <v>231</v>
       </c>
       <c r="R14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="S14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U14" s="7">
         <v>1</v>
       </c>
       <c r="V14" s="6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="W14" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X14" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="15" spans="1:24" ht="71.25">
+    <row r="15" spans="1:24" ht="142.5">
       <c r="A15" s="2" t="s">
         <v>89</v>
       </c>
@@ -2059,46 +2056,46 @@
         <v>96</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="M15" s="2" t="s">
         <v>88</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="P15" t="s">
         <v>213</v>
       </c>
       <c r="Q15" t="s">
-        <v>232</v>
+        <v>305</v>
       </c>
       <c r="R15" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S15" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U15" s="7">
         <v>1</v>
       </c>
       <c r="V15" s="6" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="W15" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X15" s="6" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="57">
+    <row r="16" spans="1:24" ht="142.5">
       <c r="A16" s="2" t="s">
         <v>97</v>
       </c>
@@ -2133,7 +2130,7 @@
         <v>103</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="M16" s="2" t="s">
         <v>42</v>
@@ -2148,31 +2145,31 @@
         <v>214</v>
       </c>
       <c r="Q16" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="R16" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="S16" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="T16" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U16" s="7">
         <v>1</v>
       </c>
       <c r="V16" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="W16" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X16" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="17" spans="1:24" ht="57">
+    <row r="17" spans="1:24" ht="142.5">
       <c r="A17" s="2" t="s">
         <v>104</v>
       </c>
@@ -2207,7 +2204,7 @@
         <v>110</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="M17" s="2" t="s">
         <v>111</v>
@@ -2222,31 +2219,31 @@
         <v>215</v>
       </c>
       <c r="Q17" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="R17" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S17" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U17" s="7">
         <v>1</v>
       </c>
       <c r="V17" s="6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="W17" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X17" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="18" spans="1:24" ht="57">
+    <row r="18" spans="1:24" ht="142.5">
       <c r="A18" s="2" t="s">
         <v>112</v>
       </c>
@@ -2281,7 +2278,7 @@
         <v>119</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="M18" s="2" t="s">
         <v>120</v>
@@ -2296,31 +2293,31 @@
         <v>119</v>
       </c>
       <c r="Q18" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R18" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S18" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U18" s="7">
         <v>1</v>
       </c>
       <c r="V18" s="6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="W18" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X18" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="19" spans="1:24" ht="57">
+    <row r="19" spans="1:24" ht="142.5">
       <c r="A19" s="2" t="s">
         <v>121</v>
       </c>
@@ -2370,31 +2367,31 @@
         <v>127</v>
       </c>
       <c r="Q19" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="R19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S19" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U19" s="7">
         <v>1</v>
       </c>
       <c r="V19" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="W19" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X19" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="20" spans="1:24" ht="57">
+    <row r="20" spans="1:24" ht="142.5">
       <c r="A20" s="2" t="s">
         <v>130</v>
       </c>
@@ -2444,28 +2441,28 @@
         <v>216</v>
       </c>
       <c r="Q20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="R20" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S20" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U20" s="7">
         <v>1</v>
       </c>
       <c r="V20" s="6" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="W20" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X20" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="178.5">
@@ -2518,31 +2515,31 @@
         <v>217</v>
       </c>
       <c r="Q21" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="R21" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="S21" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="T21" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U21" s="7">
         <v>0.5</v>
       </c>
       <c r="V21" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="W21" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X21" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="22" spans="1:24" ht="57">
+    <row r="22" spans="1:24" ht="142.5">
       <c r="A22" s="2" t="s">
         <v>145</v>
       </c>
@@ -2577,7 +2574,7 @@
         <v>152</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="M22" s="2" t="s">
         <v>153</v>
@@ -2592,28 +2589,28 @@
         <v>218</v>
       </c>
       <c r="Q22" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="R22" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S22" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T22" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U22" s="7">
         <v>1</v>
       </c>
       <c r="V22" s="6" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="W22" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X22" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="23" spans="1:24" ht="178.5">
@@ -2651,7 +2648,7 @@
         <v>202</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="M23" s="2" t="s">
         <v>81</v>
@@ -2666,31 +2663,31 @@
         <v>219</v>
       </c>
       <c r="Q23" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="R23" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="S23" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="T23" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U23" s="7">
         <v>1</v>
       </c>
       <c r="V23" s="6" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="W23" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X23" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="24" spans="1:24" ht="57">
+    <row r="24" spans="1:24" ht="142.5">
       <c r="A24" s="2" t="s">
         <v>161</v>
       </c>
@@ -2740,31 +2737,31 @@
         <v>220</v>
       </c>
       <c r="Q24" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="R24" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="S24" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="T24" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="U24" s="7">
         <v>0</v>
       </c>
       <c r="V24" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="W24" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X24" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="57">
+    <row r="25" spans="1:24" ht="142.5">
       <c r="A25" s="2" t="s">
         <v>170</v>
       </c>
@@ -2814,31 +2811,31 @@
         <v>220</v>
       </c>
       <c r="Q25" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="R25" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="S25" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T25" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U25" s="7">
         <v>0.5</v>
       </c>
       <c r="V25" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="W25" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X25" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
-    <row r="26" spans="1:24" ht="57">
+    <row r="26" spans="1:24" ht="142.5">
       <c r="A26" s="2" t="s">
         <v>179</v>
       </c>
@@ -2888,28 +2885,28 @@
         <v>221</v>
       </c>
       <c r="Q26" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="R26" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S26" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="T26" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="U26" s="7">
         <v>0</v>
       </c>
       <c r="V26" s="6" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="W26" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X26" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="27" spans="1:24" ht="178.5">
@@ -2947,7 +2944,7 @@
         <v>203</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="M27" s="2" t="s">
         <v>195</v>
@@ -2962,28 +2959,28 @@
         <v>222</v>
       </c>
       <c r="Q27" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="R27" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="S27" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="T27" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U27" s="7">
         <v>1</v>
       </c>
       <c r="V27" s="6" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="W27" s="6" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="X27" s="6" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>